<commit_message>
KLEE test suite: close + helper functions (TODO: update global makefile with newly tested syscall)
</commit_message>
<xml_diff>
--- a/individual_Tests/chmod/chmod_test_results.xlsx
+++ b/individual_Tests/chmod/chmod_test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Masters\Tests\initial_tests\individual_Tests\chmod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEAFAE65-3864-4689-BEC7-CE49D8359886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B43BE3-5F18-4576-B6AB-D2D9EBA732B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,10 +238,10 @@
     <t>Patched</t>
   </si>
   <si>
-    <t>Yes, d887486</t>
-  </si>
-  <si>
     <t>⚠ chmod() concretizes the symbolic st_mode in KLEE's sym-files. T08-T11 prove chmod actually affects subsequent open() permission checks. T13 proves chmod gives deterministic single-path execution (kinda).</t>
+  </si>
+  <si>
+    <t>Yes, d887486, will break open()</t>
   </si>
 </sst>
 </file>
@@ -724,7 +724,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -979,7 +979,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="8"/>
     </row>
-    <row r="12" spans="1:9" ht="39.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>48</v>
       </c>
@@ -1003,10 +1003,10 @@
         <v>69</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="39.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>51</v>
       </c>
@@ -1030,7 +1030,7 @@
         <v>69</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="26.25" thickTop="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KLEE test suite: added dup/dup2 tests, global makefile with all testes syscalls, overall findings, removed some verbose + helper funcions
</commit_message>
<xml_diff>
--- a/individual_Tests/chmod/chmod_test_results.xlsx
+++ b/individual_Tests/chmod/chmod_test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Masters\Tests\initial_tests\individual_Tests\chmod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B43BE3-5F18-4576-B6AB-D2D9EBA732B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271FEF38-4F4A-4FCD-945D-743D812AA299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,10 +238,10 @@
     <t>Patched</t>
   </si>
   <si>
-    <t>⚠ chmod() concretizes the symbolic st_mode in KLEE's sym-files. T08-T11 prove chmod actually affects subsequent open() permission checks. T13 proves chmod gives deterministic single-path execution (kinda).</t>
-  </si>
-  <si>
     <t>Yes, d887486, will break open()</t>
+  </si>
+  <si>
+    <t>⚠ chmod() concretizes the symbolic st_mode in KLEE's sym-files. T08-T11 prove chmod actually affects subsequent open() permission checks. T13 "proves" chmod gives deterministic single-path execution (kinda).</t>
   </si>
 </sst>
 </file>
@@ -724,7 +724,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -1003,7 +1003,7 @@
         <v>69</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1030,7 +1030,7 @@
         <v>69</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="26.25" thickTop="1" x14ac:dyDescent="0.25">

</xml_diff>